<commit_message>
Update Lab 01 POA&M:
status, marking, control mapping
</commit_message>
<xml_diff>
--- a/01-Vulnerability-Assessment/POA&M-Homelab-Jul2-2026.xlsx
+++ b/01-Vulnerability-Assessment/POA&M-Homelab-Jul2-2026.xlsx
@@ -620,7 +620,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>System: Cybersecurity Homelab | Owner: Gideon Sarfo-Nyantakyi | Classification: UNCLASSIFIED // FOR OFFICIAL USE ONLY</t>
+          <t>System: Cybersecurity Homelab | Owner: Gideon Sarfo-Nyantakyi | Personal lab — public portfolio document | Updated: September 30, 2026</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t>Gideon Sarfo-Nyantakyi, GRC Analyst</t>
+          <t>Gideon Sarfo-Nyantakyi</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
@@ -849,7 +849,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1">
+    <row r="7" ht="165" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
         <is>
           <t>POA&amp;M-002</t>
@@ -868,7 +868,7 @@
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>RA-5(1) – Vulnerability Scanning | Authenticated Scans
+          <t>RA-5(5) – Vulnerability Monitoring and Scanning | Privileged Access (authenticated scans)
 CA-7 – Continuous Monitoring</t>
         </is>
       </c>
@@ -889,22 +889,18 @@
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>August 2, 2026</t>
+          <t>October 31, 2026 (re-baselined; originally August 2, 2026)</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>1. Research SSH credential-based scanning in OpenVAS
-2. Configure scan credentials in GVM
-3. Re-run authenticated scan
-4. Document results</t>
+          <t>Changed September 30, 2026: original milestones (July 15 – August 2, 2026) were missed. Re-baselined to October 31, 2026 to align with Lab 03.</t>
         </is>
       </c>
       <c r="J7" s="10" t="inlineStr">
         <is>
-          <t>Milestone 1: Research authenticated scan config – July 15, 2026
-Milestone 2: Configure credentials – July 22, 2026
-Milestone 3: Run authenticated scan – August 2, 2026</t>
+          <t>Original (missed): M1 Research authenticated scan config – July 15, 2026; M2 Configure credentials – July 22, 2026; M3 Run authenticated scan – August 2, 2026
+Revised: Configure SSH credentials in GVM, run authenticated scan, and document results – October 31, 2026</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
@@ -915,7 +911,7 @@
       </c>
       <c r="L7" s="11" t="inlineStr">
         <is>
-          <t>OPEN – In Progress</t>
+          <t>OPEN – Overdue, re-baselined</t>
         </is>
       </c>
       <c r="M7" s="10" t="inlineStr">
@@ -930,7 +926,7 @@
       </c>
       <c r="O7" s="10" t="inlineStr"/>
     </row>
-    <row r="8" ht="90" customHeight="1">
+    <row r="8" ht="165" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>POA&amp;M-003</t>
@@ -956,8 +952,8 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Home Network Range
-192.168.1.0/24 (estimated)</t>
+          <t>Homelab assessment scope
+(originally planned: home network 192.168.1.0/24)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -977,17 +973,13 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>1. Reconfigure VirtualBox network adapter to Bridged mode
-2. Identify home network IP range
-3. Run full network scan
-4. Build asset inventory from results</t>
+          <t>Changed September 29, 2026: approach changed from a bridged home-network scan to an isolated lab network (Lab 02), to avoid exposing an intentionally vulnerable VM and scanning devices outside sole authority.</t>
         </is>
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>Milestone 1: Configure bridged networking – July 16, 2026
-Milestone 2: Run network-wide scan – August 2, 2026
-Milestone 3: Complete asset inventory – August 16, 2026</t>
+          <t>Original: M1 Configure bridged networking – July 16, 2026; M2 Run network-wide scan – August 2, 2026; M3 Complete asset inventory – August 16, 2026
+Actual: Isolated "GRC-Lab" network, target VM added, full scan and CM-8 inventory completed – September 29, 2026</t>
         </is>
       </c>
       <c r="K8" s="7" t="inlineStr">
@@ -996,9 +988,9 @@
 OpenVAS/GVM</t>
         </is>
       </c>
-      <c r="L8" s="12" t="inlineStr">
-        <is>
-          <t>OPEN – Planned</t>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>CLOSED – Completed via Lab 02</t>
         </is>
       </c>
       <c r="M8" s="7" t="inlineStr">
@@ -1008,10 +1000,14 @@
       </c>
       <c r="N8" s="7" t="inlineStr">
         <is>
-          <t>Expanding scan to full home network will produce richer portfolio artifacts including asset inventory, network diagram, and multi-host vulnerability findings aligned to CM-8 and RA-5.</t>
-        </is>
-      </c>
-      <c r="O8" s="7" t="inlineStr"/>
+          <t>Closed by Lab 02 (02-Network-Enumeration): 4 components discovered and inventoried, 30 services enumerated on the target, findings tracked as POA&amp;M-004 to POA&amp;M-012.</t>
+        </is>
+      </c>
+      <c r="O8" s="7" t="inlineStr">
+        <is>
+          <t>September 29, 2026</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1047,7 +1043,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>System: Cybersecurity Homelab | Scan Date: July 2, 2026 | Scanner: OpenVAS GVM 26.17.0</t>
+          <t>System: Cybersecurity Homelab | Scan Date: July 2, 2026 | Scanner: OpenVAS GVM 26.17.0 | Updated: September 30, 2026</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1196,7 @@
         </is>
       </c>
       <c r="B11" s="16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
@@ -1209,7 +1205,7 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>POA&amp;M-002 and POA&amp;M-003</t>
+          <t>POA&amp;M-002 (overdue; re-baselined to October 31, 2026)</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1216,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C12" s="19" t="inlineStr">
         <is>
@@ -1229,7 +1225,7 @@
       </c>
       <c r="D12" s="18" t="inlineStr">
         <is>
-          <t>POA&amp;M-001</t>
+          <t>POA&amp;M-001, POA&amp;M-003</t>
         </is>
       </c>
     </row>
@@ -1244,14 +1240,14 @@
           <t>1 Host</t>
         </is>
       </c>
-      <c r="C13" s="22" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>EXPANDED</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>Expanding to full network in POA&amp;M-003</t>
+          <t>Scope expanded in Lab 02 (isolated network, 4 components); POA&amp;M-003 closed</t>
         </is>
       </c>
     </row>
@@ -1288,14 +1284,14 @@
           <t>August 2, 2026</t>
         </is>
       </c>
-      <c r="C15" s="20" t="inlineStr">
-        <is>
-          <t>SCHEDULED</t>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>MISSED</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>Per continuous monitoring plan</t>
+          <t>Follow-up scan did not occur; to be performed after Lab 03</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1303,7 @@
       </c>
       <c r="B16" s="18" t="inlineStr">
         <is>
-          <t>RA-5, CA-7, RA-3, CM-8</t>
+          <t>RA-5, RA-5(5), CA-7, RA-3, CM-8</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">

</xml_diff>